<commit_message>
Stage pending changes: scenario updates, branding assets, DLEMBA course move
- Updated BUS-314 scenario workbooks (AAPL, CAT, MSFT, WMT, XOM)
- Moved BUS-620-DLEMBA-Micro-And-Macro-Economics into courses/
- Added FreshSends branding assets (design-system-fresh-sends.html,
  freshsends-design.json)
- Added shidler-finance-light template variants (.potx, .pptx)
- Updated FIN-321 scenario 2 FX hedging memo

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/courses/BUS-314-International-Corporate-Finance/accounting-ratios/_scenarios/BUS314_AAPL_Scenario.xlsx
+++ b/courses/BUS-314-International-Corporate-Finance/accounting-ratios/_scenarios/BUS314_AAPL_Scenario.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\shidler\BUS-314-International-Corporate-Finance\accounting-ratios\_scenarios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\shidler\courses\BUS-314-International-Corporate-Finance\accounting-ratios\_scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C84E602-EB6E-44A5-B290-B863DA07D30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDDF135-5D5E-44BB-BF78-47C55575DD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Balance Sheet" sheetId="1" r:id="rId1"/>
@@ -210,7 +210,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Adam Stauffer:</t>
         </r>
@@ -219,7 +219,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Links to Income Statement net income. Source: Apple 10-K FY2024</t>
@@ -234,7 +234,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Adam Stauffer:</t>
         </r>
@@ -243,7 +243,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Change in accounts receivable per Apple 10-K FY2024 cash flow statement</t>
@@ -258,7 +258,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Adam Stauffer:</t>
         </r>
@@ -267,7 +267,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Change in inventories per Apple 10-K FY2024 cash flow statement</t>
@@ -282,7 +282,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Change in other current and non-current assets (excluding vendor non-trade receivables). Source: Apple 10-K FY2024 cash flow statement</t>
         </r>
@@ -296,7 +296,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Adam Stauffer:</t>
         </r>
@@ -305,7 +305,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Increase in other current and non-current liabilities. Source: Apple 10-K FY2024</t>
@@ -320,7 +320,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Adam Stauffer:</t>
         </r>
@@ -329,7 +329,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Net proceeds from marketable securities: maturities (51,211) + sales (11,135) - purchases (48,656) = 13,690. Source: Apple 10-K FY2024</t>
@@ -344,7 +344,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Adam Stauffer:</t>
         </r>
@@ -353,7 +353,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Repayments of term debt. Source: Apple 10-K FY2024</t>
@@ -368,7 +368,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Adam Stauffer:</t>
         </r>
@@ -377,7 +377,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Net proceeds from commercial paper. Source: Apple 10-K FY2024</t>
@@ -392,7 +392,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Adam Stauffer:</t>
         </r>
@@ -401,7 +401,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Taxes on share settlements (-5,441) + other (-361). Source: Apple 10-K FY2024</t>
@@ -1256,7 +1256,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1396,19 +1396,6 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="17">
@@ -1745,10 +1732,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1940,7 +1923,9 @@
   <we:alternateReferences>
     <we:reference id="WA200009404" version="1.0.0.5" store="" storeType="OMEX"/>
   </we:alternateReferences>
-  <we:properties/>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;cee1255c-bb48-4c9e-98eb-74b1a2986dcb&quot;"/>
+  </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </we:webextension>
@@ -2456,7 +2441,8 @@
         <v>11445</v>
       </c>
       <c r="D7" s="25">
-        <v>2.9268479803598101E-2</v>
+        <f>IF(C$4=0,0,C7/C$4)</f>
+        <v>2.9268479803598143E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -2504,6 +2490,7 @@
         <v>3931</v>
       </c>
       <c r="D11" s="25">
+        <f>IF(C$4=0,0,C11/C$4)</f>
         <v>1.00528085721227E-2</v>
       </c>
     </row>
@@ -2539,7 +2526,8 @@
         <v>29749</v>
       </c>
       <c r="D14" s="25">
-        <v>7.6077588962624801E-2</v>
+        <f>IF(C$4=0,0,C14/C$4)</f>
+        <v>7.6077588962624829E-2</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -2692,6 +2680,7 @@
         <v>54</v>
       </c>
       <c r="C6" s="22">
+        <f>'Income Statement'!C7</f>
         <v>11445</v>
       </c>
       <c r="D6" s="27" t="s">

</xml_diff>